<commit_message>
notas 2eval 1eso metidas con cambios oficiales tras reunion claustro 2eval
</commit_message>
<xml_diff>
--- a/matematicas_1ESOA/notas/E1A_eval2.xlsx
+++ b/matematicas_1ESOA/notas/E1A_eval2.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="81">
   <si>
     <t>HOJA DE CÁLCULO PARA GENERAR UN ACTILLA DE EVALUACIÓN</t>
   </si>
@@ -711,6 +711,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -722,15 +731,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1016,10 +1016,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1349,16 +1345,16 @@
       </c>
     </row>
     <row r="8" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="45" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="45"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="45"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C9" s="2" t="s">
@@ -1376,16 +1372,16 @@
       </c>
     </row>
     <row r="15" spans="2:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="42" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
+      <c r="B15" s="45" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="45"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="45"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
@@ -1408,16 +1404,16 @@
       </c>
     </row>
     <row r="22" spans="2:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="42" t="s">
+      <c r="B22" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="42"/>
-      <c r="D22" s="42"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="42"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="42"/>
+      <c r="C22" s="45"/>
+      <c r="D22" s="45"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="45"/>
+      <c r="G22" s="45"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="45"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N23" s="4" t="s">
@@ -2152,11 +2148,11 @@
         <f t="shared" si="3"/>
         <v>5.0999999999999996</v>
       </c>
-      <c r="W9" s="39" t="s">
+      <c r="W9" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="X9" s="39"/>
-      <c r="Y9" s="39"/>
+      <c r="X9" s="42"/>
+      <c r="Y9" s="42"/>
     </row>
     <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="27">
@@ -2226,9 +2222,9 @@
         <f t="shared" si="3"/>
         <v>7.9</v>
       </c>
-      <c r="W10" s="39"/>
-      <c r="X10" s="39"/>
-      <c r="Y10" s="39"/>
+      <c r="W10" s="42"/>
+      <c r="X10" s="42"/>
+      <c r="Y10" s="42"/>
     </row>
     <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="19">
@@ -2298,9 +2294,9 @@
         <f t="shared" si="3"/>
         <v>8.8000000000000007</v>
       </c>
-      <c r="W11" s="39"/>
-      <c r="X11" s="39"/>
-      <c r="Y11" s="39"/>
+      <c r="W11" s="42"/>
+      <c r="X11" s="42"/>
+      <c r="Y11" s="42"/>
     </row>
     <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="27">
@@ -2370,11 +2366,11 @@
         <f t="shared" si="3"/>
         <v>7.9</v>
       </c>
-      <c r="W12" s="40" t="s">
+      <c r="W12" s="43" t="s">
         <v>74</v>
       </c>
-      <c r="X12" s="40"/>
-      <c r="Y12" s="40"/>
+      <c r="X12" s="43"/>
+      <c r="Y12" s="43"/>
     </row>
     <row r="13" spans="1:25" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="19">
@@ -2444,9 +2440,9 @@
         <f t="shared" si="3"/>
         <v>4.3</v>
       </c>
-      <c r="W13" s="40"/>
-      <c r="X13" s="40"/>
-      <c r="Y13" s="40"/>
+      <c r="W13" s="43"/>
+      <c r="X13" s="43"/>
+      <c r="Y13" s="43"/>
     </row>
     <row r="14" spans="1:25" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="27">
@@ -2458,7 +2454,7 @@
       <c r="C14" s="38">
         <v>5</v>
       </c>
-      <c r="D14" s="43">
+      <c r="D14" s="39">
         <v>7</v>
       </c>
       <c r="E14" s="38">
@@ -2516,9 +2512,9 @@
         <f t="shared" si="3"/>
         <v>6.7</v>
       </c>
-      <c r="W14" s="40"/>
-      <c r="X14" s="40"/>
-      <c r="Y14" s="40"/>
+      <c r="W14" s="43"/>
+      <c r="X14" s="43"/>
+      <c r="Y14" s="43"/>
     </row>
     <row r="15" spans="1:25" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="19">
@@ -2588,11 +2584,11 @@
         <f t="shared" si="3"/>
         <v>6.1</v>
       </c>
-      <c r="W15" s="41" t="s">
+      <c r="W15" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="X15" s="41"/>
-      <c r="Y15" s="41"/>
+      <c r="X15" s="44"/>
+      <c r="Y15" s="44"/>
     </row>
     <row r="16" spans="1:25" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="27">
@@ -3018,7 +3014,7 @@
       <c r="C22" s="38">
         <v>8</v>
       </c>
-      <c r="D22" s="45">
+      <c r="D22" s="41">
         <v>7</v>
       </c>
       <c r="E22" s="38">
@@ -3156,7 +3152,7 @@
       <c r="C24" s="38">
         <v>7</v>
       </c>
-      <c r="D24" s="43">
+      <c r="D24" s="39">
         <v>4</v>
       </c>
       <c r="E24" s="38">
@@ -3225,10 +3221,10 @@
       <c r="C25" s="37">
         <v>8</v>
       </c>
-      <c r="D25" s="44">
-        <v>5</v>
-      </c>
-      <c r="E25" s="44">
+      <c r="D25" s="40">
+        <v>5</v>
+      </c>
+      <c r="E25" s="40">
         <v>6</v>
       </c>
       <c r="F25" s="37">
@@ -3297,7 +3293,7 @@
       <c r="D26" s="38">
         <v>8</v>
       </c>
-      <c r="E26" s="43">
+      <c r="E26" s="39">
         <v>7</v>
       </c>
       <c r="F26" s="28" t="s">

</xml_diff>